<commit_message>
feat: harden campaign automation and product curation
Adds inventory safety (fresh BigCommerce rechecks pre-export/pre-Klaviyo),
exact SS/RDD product-count rules, quality/depth-weighted category
allocation replacing equal round-robin curation, restored SS product-card
descriptions sourced from verified BigCommerce data with hardened QA
(empty/duplicate/placeholder descriptions now block), and a function-aware
product-grid pairing layer (same base family > same function >
complementary > shared stem > category > fallback) shared across all
brands. Includes theme-relevance/coherence QA, hero and support-banner
resolvers, ImageKit hosting pipeline, natural-language campaign generation,
and associated test coverage.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Calendar Campaign/RDD Campaign Calendar.xlsx
+++ b/Calendar Campaign/RDD Campaign Calendar.xlsx
@@ -807,28 +807,28 @@
         <v>RDD-2026-36</v>
       </c>
       <c r="B10" t="str">
-        <v>Father's Day Workplace Comfort Sale</v>
+        <v>Father's Day: Click &amp; Collect Home Office Gifts</v>
       </c>
       <c r="C10" t="str">
-        <v>Promotional sale</v>
+        <v>Holiday gifting</v>
       </c>
       <c r="D10" t="str">
-        <v>Give Dad the Gift of Workplace Comfort</v>
+        <v>Father's Day is Sunday. Collect Dad's Gift Locally</v>
       </c>
       <c r="E10">
         <v>46261</v>
       </c>
       <c r="F10" t="str">
-        <v>Sit Stand Desks, Ergonomic Chairs</v>
+        <v>Ergonomic Office Chairs, Sit-Stand Desks, Desk Accessories, Storage</v>
       </c>
       <c r="G10" t="str">
-        <v>15% off selected ergonomic workplace products.</v>
+        <v>Father's Day + LOCAL PICKUP. Skip the delivery wait, Pickup from the Sydney warehouse (order online, collect in store). Ergonomic chairs, sit-stand desks, desk accessories. CTA: Shop Father's Day Gifts to /products/, choose Pickup at checkout. No discount.</v>
       </c>
       <c r="H10" t="str">
-        <v>DADDEALS15</v>
+        <v/>
       </c>
       <c r="I10" t="str">
-        <v>15% off sit stand desks &amp; chairs</v>
+        <v/>
       </c>
       <c r="J10" t="str">
         <v>warm, celebratory, gifting</v>
@@ -843,7 +843,7 @@
         <v>pending</v>
       </c>
       <c r="O10" t="str">
-        <v xml:space="preserve"> </v>
+        <v>Revised to Local Pickup focus per Bruce. Pickup VERIFIED (retaildisplaydirect.com.au/shipping-returns). Draft v5: removed the two-hours wording and the Why RDD trust section; relabelled Click &amp; Collect to Pickup. Klaviyo draft updated. Intended send today 1pm.</v>
       </c>
     </row>
     <row r="11">

</xml_diff>